<commit_message>
Update project files and latest validation outputs
</commit_message>
<xml_diff>
--- a/01_Raw_Data/Interest_Rates/Weighted Average Lending Rate.xlsx
+++ b/01_Raw_Data/Interest_Rates/Weighted Average Lending Rate.xlsx
@@ -1,16 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
+  <workbookPr showInkAnnotation="0" autoCompressPictures="0" defaultThemeVersion="166925"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_D8E9CBBB4943957784D962D28111B65052F43767" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Sector Wise" sheetId="1" r:id="rId1"/>
     <sheet name="Credit Range Wise" sheetId="2" r:id="rId2"/>
     <sheet name="Type of Account Wise" sheetId="3" r:id="rId3"/>
   </sheets>
+  <calcPr calcId="0" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="30">
+  <si>
+    <t>Weighted average lending rate of SCBs for all loans and for major sectors - as on 31st March</t>
+  </si>
+  <si>
+    <t>(Per cent)</t>
+  </si>
   <si>
     <t>Year</t>
   </si>
@@ -42,13 +60,7 @@
     <t>WALR</t>
   </si>
   <si>
-    <t>Weighted average lending rate of SCBs for all loans and for major sectors - as on 31st March</t>
-  </si>
-  <si>
-    <t>(Per cent)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source: Basic Statistical Return (BSR) -1 of Scheduled Commercial Banks in India
+    <t>Source: Basic Statistical Return (BSR) -1 of Scheduled Commercial Banks in India
 (Link:- www.rbi.org.in -&gt; Publications -&gt; Annual -&gt; Basic Stattistical Returns of Scheduled Commercial Banks in India).
 Note:-
 Related to accounts with credit limit more than Rupees 25,000 till 1998 and more than Rupees 200,000 till 2012 and for all accounts thereafter.
@@ -56,6 +68,9 @@
 WALR: Weighted average nominal lending rate.
 The WALR data are exclusive of foreign and inland bills purchased and discounted.
 Amount outstanding is taken as the weight for calculating average lending rates.</t>
+  </si>
+  <si>
+    <t>Weighted average lending rate of SCBs according to credit limit range - as on 31st March</t>
   </si>
   <si>
     <t>`100 million &lt; Credit Limit &lt;= `1 billion</t>
@@ -82,7 +97,7 @@
     <t>NA</t>
   </si>
   <si>
-    <t>Weighted average lending rate of SCBs according to credit limit range - as on 31st March</t>
+    <t>Weighted average lending rate of SCBs according to type of account - as on 31st March</t>
   </si>
   <si>
     <t>Cash Credit</t>
@@ -105,17 +120,13 @@
   <si>
     <t>All accounts</t>
   </si>
-  <si>
-    <t>Weighted average lending rate of SCBs according to type of account - as on 31st March</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="172" formatCode="0"/>
-    <numFmt numFmtId="173" formatCode="0.0;\-0.0;0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0;\-0.0;0"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -125,37 +136,37 @@
     </font>
     <font>
       <sz val="9"/>
-      <color rgb="00333333"/>
+      <color rgb="FF333333"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
-      <color rgb="00333333"/>
+      <color rgb="FF333333"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
-      <color rgb="00488AC7"/>
+      <color rgb="FF488AC7"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
-      <color rgb="00333333"/>
+      <color rgb="FF333333"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <sz val="8"/>
-      <color rgb="00333333"/>
+      <color rgb="FF333333"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -164,10 +175,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125">
-        <fgColor rgb="00000000"/>
-        <bgColor rgb="00000000"/>
-      </patternFill>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -198,25 +206,25 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </right>
       <top/>
       <bottom/>
@@ -224,14 +232,14 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color rgb="00000000"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -239,167 +247,478 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom"/>
+  <cellXfs count="13">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="3" fillId="4" borderId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom"/>
+    <xf numFmtId="1" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="173" fontId="1" fillId="4" borderId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="173" fontId="1" fillId="2" borderId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="172" fontId="3" fillId="4" borderId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom"/>
+    <xf numFmtId="1" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="173" fontId="1" fillId="4" borderId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="bottom"/>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1" horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4472C4"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O32"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B1:P32"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.67767866666667" customWidth="1"/>
-    <col min="2" max="2" width="10.7125106666667" customWidth="1"/>
-    <col min="3" max="3" width="10.685892" customWidth="1"/>
-    <col min="4" max="4" width="12.7089106666667" customWidth="1"/>
-    <col min="5" max="5" width="10.6820893333333" customWidth="1"/>
-    <col min="6" max="6" width="12.7089106666667" customWidth="1"/>
-    <col min="7" max="7" width="10.6820893333333" customWidth="1"/>
-    <col min="8" max="8" width="12.7089106666667" customWidth="1"/>
-    <col min="9" max="9" width="10.6820893333333" customWidth="1"/>
-    <col min="10" max="10" width="12.7089106666667" customWidth="1"/>
-    <col min="11" max="11" width="10.6820893333333" customWidth="1"/>
-    <col min="12" max="12" width="12.7089106666667" customWidth="1"/>
-    <col min="13" max="13" width="10.6820893333333" customWidth="1"/>
-    <col min="14" max="14" width="12.7089106666667" customWidth="1"/>
-    <col min="15" max="15" width="10.6820893333333" customWidth="1"/>
-    <col min="16" max="16" width="12.7089106666667" customWidth="1"/>
+    <col min="1" max="1" width="4.7109375" customWidth="1"/>
+    <col min="2" max="3" width="10.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="10.7109375" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" customWidth="1"/>
+    <col min="15" max="15" width="10.7109375" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="28.7982" customHeight="1"/>
-    <row r="2" s="1" customFormat="1" ht="31.4647" customHeight="1">
-      <c r="B2" s="8" t="s">
+    <row r="1" spans="2:16" s="1" customFormat="1" ht="28.7" customHeight="1"/>
+    <row r="2" spans="2:16" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="B2" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+    </row>
+    <row r="3" spans="2:16" s="1" customFormat="1" ht="14.45" customHeight="1"/>
+    <row r="4" spans="2:16" s="1" customFormat="1" ht="11.1" customHeight="1">
+      <c r="B4" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:16" s="1" customFormat="1" ht="6.95" customHeight="1"/>
+    <row r="6" spans="2:16" s="1" customFormat="1" ht="24" customHeight="1">
+      <c r="B6" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="L6" s="11"/>
+      <c r="M6" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="N6" s="11"/>
+      <c r="O6" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="P6" s="11"/>
+    </row>
+    <row r="7" spans="2:16" s="1" customFormat="1" ht="24" customHeight="1">
+      <c r="B7" s="11"/>
+      <c r="C7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-    </row>
-    <row r="3" s="1" customFormat="1" ht="14.3991" customHeight="1"/>
-    <row r="4" s="1" customFormat="1" ht="11.1993" customHeight="1">
-      <c r="B4" s="9" t="s">
+      <c r="D7" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" s="1" customFormat="1" ht="6.9329" customHeight="1"/>
-    <row r="6" s="1" customFormat="1" ht="23.9985" customHeight="1">
-      <c r="B6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="P6" s="2"/>
-    </row>
-    <row r="7" s="1" customFormat="1" ht="23.9985" customHeight="1">
-      <c r="B7" s="2"/>
-      <c r="C7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="E7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" s="1" customFormat="1" ht="19.7321" customHeight="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B8" s="3">
         <v>2014</v>
       </c>
@@ -422,7 +741,7 @@
         <v>12.3</v>
       </c>
       <c r="I8" s="4">
-        <v>8.8</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="J8" s="4">
         <v>10.7</v>
@@ -446,7 +765,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="9" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B9" s="3">
         <v>2013</v>
       </c>
@@ -457,19 +776,19 @@
         <v>10.6</v>
       </c>
       <c r="E9" s="5">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="F9" s="5">
         <v>12.4</v>
       </c>
       <c r="G9" s="5">
-        <v>40.8</v>
+        <v>40.799999999999997</v>
       </c>
       <c r="H9" s="5">
         <v>12.3</v>
       </c>
       <c r="I9" s="5">
-        <v>8.8</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="J9" s="5">
         <v>10.8</v>
@@ -493,7 +812,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="10" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B10" s="3">
         <v>2012</v>
       </c>
@@ -516,7 +835,7 @@
         <v>12.8</v>
       </c>
       <c r="I10" s="4">
-        <v>8.3</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="J10" s="4">
         <v>11.1</v>
@@ -540,7 +859,7 @@
         <v>12.6</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="11" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B11" s="3">
         <v>2011</v>
       </c>
@@ -587,7 +906,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="12" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="12" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B12" s="3">
         <v>2010</v>
       </c>
@@ -610,10 +929,10 @@
         <v>10.5</v>
       </c>
       <c r="I12" s="4">
-        <v>9.7</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="J12" s="4">
-        <v>9.7</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="K12" s="4">
         <v>5</v>
@@ -634,7 +953,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="13" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="13" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B13" s="3">
         <v>2009</v>
       </c>
@@ -645,7 +964,7 @@
         <v>11</v>
       </c>
       <c r="E13" s="5">
-        <v>2.2</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="F13" s="5">
         <v>11.9</v>
@@ -681,7 +1000,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="14" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="14" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B14" s="3">
         <v>2008</v>
       </c>
@@ -728,7 +1047,7 @@
         <v>12.3</v>
       </c>
     </row>
-    <row r="15" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="15" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B15" s="3">
         <v>2007</v>
       </c>
@@ -775,7 +1094,7 @@
         <v>11.9</v>
       </c>
     </row>
-    <row r="16" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="16" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B16" s="3">
         <v>2006</v>
       </c>
@@ -822,7 +1141,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="17" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B17" s="3">
         <v>2005</v>
       </c>
@@ -869,7 +1188,7 @@
         <v>12.6</v>
       </c>
     </row>
-    <row r="18" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="18" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B18" s="3">
         <v>2004</v>
       </c>
@@ -880,7 +1199,7 @@
         <v>13</v>
       </c>
       <c r="E18" s="4">
-        <v>4.9</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="F18" s="4">
         <v>13.2</v>
@@ -916,7 +1235,7 @@
         <v>13.2</v>
       </c>
     </row>
-    <row r="19" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="19" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B19" s="3">
         <v>2003</v>
       </c>
@@ -963,7 +1282,7 @@
         <v>13.3</v>
       </c>
     </row>
-    <row r="20" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="20" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B20" s="3">
         <v>2002</v>
       </c>
@@ -986,7 +1305,7 @@
         <v>14</v>
       </c>
       <c r="I20" s="4">
-        <v>4.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="J20" s="4">
         <v>12.1</v>
@@ -1010,12 +1329,12 @@
         <v>13.7</v>
       </c>
     </row>
-    <row r="21" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="21" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B21" s="3">
         <v>2001</v>
       </c>
       <c r="C21" s="5">
-        <v>4.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="D21" s="5">
         <v>14.4</v>
@@ -1057,12 +1376,12 @@
         <v>14.1</v>
       </c>
     </row>
-    <row r="22" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="22" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B22" s="3">
         <v>2000</v>
       </c>
       <c r="C22" s="4">
-        <v>4.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="D22" s="4">
         <v>14.8</v>
@@ -1086,7 +1405,7 @@
         <v>12.5</v>
       </c>
       <c r="K22" s="4">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="L22" s="4">
         <v>15.5</v>
@@ -1104,7 +1423,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="23" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="23" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B23" s="3">
         <v>1999</v>
       </c>
@@ -1151,7 +1470,7 @@
         <v>15.4</v>
       </c>
     </row>
-    <row r="24" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="24" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B24" s="3">
         <v>1998</v>
       </c>
@@ -1198,7 +1517,7 @@
         <v>16.2</v>
       </c>
     </row>
-    <row r="25" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="25" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B25" s="3">
         <v>1997</v>
       </c>
@@ -1242,10 +1561,10 @@
         <v>100</v>
       </c>
       <c r="P25" s="5">
-        <v>16.9</v>
-      </c>
-    </row>
-    <row r="26" s="1" customFormat="1" ht="19.7321" customHeight="1">
+        <v>16.899999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B26" s="3">
         <v>1996</v>
       </c>
@@ -1274,7 +1593,7 @@
         <v>10.9</v>
       </c>
       <c r="K26" s="4">
-        <v>4.4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="L26" s="4">
         <v>16.3</v>
@@ -1289,10 +1608,10 @@
         <v>100</v>
       </c>
       <c r="P26" s="4">
-        <v>17.1</v>
-      </c>
-    </row>
-    <row r="27" s="1" customFormat="1" ht="19.7321" customHeight="1">
+        <v>17.100000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B27" s="3">
         <v>1995</v>
       </c>
@@ -1306,7 +1625,7 @@
         <v>6.9</v>
       </c>
       <c r="F27" s="5">
-        <v>16.1</v>
+        <v>16.100000000000001</v>
       </c>
       <c r="G27" s="5">
         <v>52.8</v>
@@ -1321,7 +1640,7 @@
         <v>9.6</v>
       </c>
       <c r="K27" s="5">
-        <v>4.6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="L27" s="5">
         <v>15.5</v>
@@ -1339,7 +1658,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="28" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B28" s="3">
         <v>1994</v>
       </c>
@@ -1359,13 +1678,13 @@
         <v>57.1</v>
       </c>
       <c r="H28" s="4">
-        <v>17.4</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="I28" s="4">
         <v>3.5</v>
       </c>
       <c r="J28" s="4">
-        <v>8.7</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="K28" s="4">
         <v>3.8</v>
@@ -1386,7 +1705,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="29" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="29" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B29" s="3">
         <v>1993</v>
       </c>
@@ -1400,19 +1719,19 @@
         <v>3.9</v>
       </c>
       <c r="F29" s="5">
-        <v>16.9</v>
+        <v>16.899999999999999</v>
       </c>
       <c r="G29" s="5">
         <v>58.5</v>
       </c>
       <c r="H29" s="5">
-        <v>17.9</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="I29" s="5">
         <v>3.6</v>
       </c>
       <c r="J29" s="5">
-        <v>8.3</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="K29" s="5">
         <v>3.2</v>
@@ -1433,7 +1752,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="30" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B30" s="6">
         <v>1992</v>
       </c>
@@ -1447,13 +1766,13 @@
         <v>3.6</v>
       </c>
       <c r="F30" s="7">
-        <v>16.4</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="G30" s="7">
         <v>58.7</v>
       </c>
       <c r="H30" s="7">
-        <v>17.9</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="I30" s="7">
         <v>3.4</v>
@@ -1471,7 +1790,7 @@
         <v>22.6</v>
       </c>
       <c r="N30" s="7">
-        <v>17.1</v>
+        <v>17.100000000000001</v>
       </c>
       <c r="O30" s="7">
         <v>100</v>
@@ -1480,8 +1799,8 @@
         <v>16.8</v>
       </c>
     </row>
-    <row r="31" s="1" customFormat="1" ht="6.9329" customHeight="1"/>
-    <row r="32" s="1" customFormat="1" ht="96.5273" customHeight="1">
+    <row r="31" spans="2:16" s="1" customFormat="1" ht="6.95" customHeight="1"/>
+    <row r="32" spans="2:16" s="1" customFormat="1" ht="96.6" customHeight="1">
       <c r="B32" s="10" t="s">
         <v>12</v>
       </c>
@@ -1499,6 +1818,7 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="O6:P6"/>
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="B32:M32"/>
     <mergeCell ref="B6:B7"/>
@@ -1508,135 +1828,135 @@
     <mergeCell ref="I6:J6"/>
     <mergeCell ref="K6:L6"/>
     <mergeCell ref="M6:N6"/>
-    <mergeCell ref="O6:P6"/>
   </mergeCells>
-  <pageSetup paperSize="9" scale="100" orientation="portrait"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O32"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="B1:P32"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.67767866666667" customWidth="1"/>
-    <col min="2" max="2" width="10.7125106666667" customWidth="1"/>
-    <col min="3" max="3" width="10.685892" customWidth="1"/>
-    <col min="4" max="4" width="12.7089106666667" customWidth="1"/>
-    <col min="5" max="5" width="10.6820893333333" customWidth="1"/>
-    <col min="6" max="6" width="12.7089106666667" customWidth="1"/>
-    <col min="7" max="7" width="10.6820893333333" customWidth="1"/>
-    <col min="8" max="8" width="12.7089106666667" customWidth="1"/>
-    <col min="9" max="9" width="10.6820893333333" customWidth="1"/>
-    <col min="10" max="10" width="12.7089106666667" customWidth="1"/>
-    <col min="11" max="11" width="10.6820893333333" customWidth="1"/>
-    <col min="12" max="12" width="12.7089106666667" customWidth="1"/>
-    <col min="13" max="13" width="10.6820893333333" customWidth="1"/>
-    <col min="14" max="14" width="12.7089106666667" customWidth="1"/>
-    <col min="15" max="15" width="10.6820893333333" customWidth="1"/>
-    <col min="16" max="16" width="12.7089106666667" customWidth="1"/>
+    <col min="1" max="1" width="4.7109375" customWidth="1"/>
+    <col min="2" max="3" width="10.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="10.7109375" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" customWidth="1"/>
+    <col min="15" max="15" width="10.7109375" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="28.7982" customHeight="1"/>
-    <row r="2" s="1" customFormat="1" ht="31.4647" customHeight="1">
-      <c r="B2" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-    </row>
-    <row r="3" s="1" customFormat="1" ht="14.3991" customHeight="1"/>
-    <row r="4" s="1" customFormat="1" ht="11.1993" customHeight="1">
-      <c r="B4" s="9" t="s">
+    <row r="1" spans="2:16" s="1" customFormat="1" ht="28.7" customHeight="1"/>
+    <row r="2" spans="2:16" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="B2" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+    </row>
+    <row r="3" spans="2:16" s="1" customFormat="1" ht="14.45" customHeight="1"/>
+    <row r="4" spans="2:16" s="1" customFormat="1" ht="11.1" customHeight="1">
+      <c r="B4" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:16" s="1" customFormat="1" ht="6.95" customHeight="1"/>
+    <row r="6" spans="2:16" s="1" customFormat="1" ht="34.700000000000003" customHeight="1">
+      <c r="B6" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="12"/>
+      <c r="I6" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="L6" s="12"/>
+      <c r="M6" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="P6" s="12"/>
+    </row>
+    <row r="7" spans="2:16" s="1" customFormat="1" ht="24" customHeight="1">
+      <c r="B7" s="11"/>
+      <c r="C7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" s="1" customFormat="1" ht="6.9329" customHeight="1"/>
-    <row r="6" s="1" customFormat="1" ht="34.6645" customHeight="1">
-      <c r="B6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="P6" s="11"/>
-    </row>
-    <row r="7" s="1" customFormat="1" ht="23.9985" customHeight="1">
-      <c r="B7" s="2"/>
-      <c r="C7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="E7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" s="1" customFormat="1" ht="19.7321" customHeight="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B8" s="3">
         <v>2014</v>
       </c>
@@ -1665,13 +1985,13 @@
         <v>12</v>
       </c>
       <c r="K8" s="4">
-        <v>32.8</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="L8" s="4">
         <v>11.5</v>
       </c>
       <c r="M8" s="4">
-        <v>600000e-6</v>
+        <v>0.6</v>
       </c>
       <c r="N8" s="4">
         <v>12.3</v>
@@ -1683,7 +2003,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="9" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B9" s="3">
         <v>2013</v>
       </c>
@@ -1706,7 +2026,7 @@
         <v>12.1</v>
       </c>
       <c r="I9" s="5">
-        <v>8.3</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="J9" s="5">
         <v>11.6</v>
@@ -1730,7 +2050,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="10" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B10" s="3">
         <v>2012</v>
       </c>
@@ -1753,10 +2073,10 @@
         <v>12.6</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K10" s="4">
         <v>34.6</v>
@@ -1765,10 +2085,10 @@
         <v>11.8</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O10" s="4">
         <v>100</v>
@@ -1777,7 +2097,7 @@
         <v>12.6</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="11" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B11" s="3">
         <v>2011</v>
       </c>
@@ -1800,10 +2120,10 @@
         <v>11.8</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K11" s="5">
         <v>33</v>
@@ -1812,10 +2132,10 @@
         <v>10.4</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O11" s="5">
         <v>100</v>
@@ -1824,7 +2144,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="12" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="12" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B12" s="3">
         <v>2010</v>
       </c>
@@ -1847,22 +2167,22 @@
         <v>11.2</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K12" s="4">
         <v>28.5</v>
       </c>
       <c r="L12" s="4">
-        <v>9.3</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N12" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O12" s="4">
         <v>100</v>
@@ -1871,7 +2191,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="13" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="13" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B13" s="3">
         <v>2009</v>
       </c>
@@ -1894,10 +2214,10 @@
         <v>12.1</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K13" s="5">
         <v>26.6</v>
@@ -1906,10 +2226,10 @@
         <v>10.4</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N13" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O13" s="5">
         <v>100</v>
@@ -1918,7 +2238,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="14" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="14" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B14" s="3">
         <v>2008</v>
       </c>
@@ -1941,10 +2261,10 @@
         <v>12.3</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K14" s="4">
         <v>22.2</v>
@@ -1953,10 +2273,10 @@
         <v>12.5</v>
       </c>
       <c r="M14" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N14" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O14" s="4">
         <v>100</v>
@@ -1965,7 +2285,7 @@
         <v>12.3</v>
       </c>
     </row>
-    <row r="15" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="15" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B15" s="3">
         <v>2007</v>
       </c>
@@ -1988,10 +2308,10 @@
         <v>11.4</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K15" s="5">
         <v>20.2</v>
@@ -2000,10 +2320,10 @@
         <v>12.1</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N15" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O15" s="5">
         <v>100</v>
@@ -2012,7 +2332,7 @@
         <v>11.9</v>
       </c>
     </row>
-    <row r="16" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="16" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B16" s="3">
         <v>2006</v>
       </c>
@@ -2035,10 +2355,10 @@
         <v>11.3</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K16" s="4">
         <v>20.2</v>
@@ -2047,10 +2367,10 @@
         <v>12.2</v>
       </c>
       <c r="M16" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N16" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O16" s="4">
         <v>100</v>
@@ -2059,7 +2379,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="17" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B17" s="3">
         <v>2005</v>
       </c>
@@ -2076,16 +2396,16 @@
         <v>13</v>
       </c>
       <c r="G17" s="5">
-        <v>33.3</v>
+        <v>33.299999999999997</v>
       </c>
       <c r="H17" s="5">
         <v>11.9</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K17" s="5">
         <v>18.2</v>
@@ -2094,10 +2414,10 @@
         <v>12.4</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N17" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O17" s="5">
         <v>100</v>
@@ -2106,7 +2426,7 @@
         <v>12.6</v>
       </c>
     </row>
-    <row r="18" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="18" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B18" s="3">
         <v>2004</v>
       </c>
@@ -2129,22 +2449,22 @@
         <v>13.4</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K18" s="4">
-        <v>16.6</v>
+        <v>16.600000000000001</v>
       </c>
       <c r="L18" s="4">
         <v>12.1</v>
       </c>
       <c r="M18" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N18" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O18" s="4">
         <v>100</v>
@@ -2153,7 +2473,7 @@
         <v>13.2</v>
       </c>
     </row>
-    <row r="19" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="19" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B19" s="3">
         <v>2003</v>
       </c>
@@ -2176,10 +2496,10 @@
         <v>13.7</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K19" s="5">
         <v>19.8</v>
@@ -2188,10 +2508,10 @@
         <v>12.3</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N19" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O19" s="5">
         <v>100</v>
@@ -2200,7 +2520,7 @@
         <v>13.3</v>
       </c>
     </row>
-    <row r="20" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="20" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B20" s="3">
         <v>2002</v>
       </c>
@@ -2223,10 +2543,10 @@
         <v>14.4</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K20" s="4">
         <v>21.4</v>
@@ -2235,10 +2555,10 @@
         <v>12.3</v>
       </c>
       <c r="M20" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N20" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O20" s="4">
         <v>100</v>
@@ -2247,7 +2567,7 @@
         <v>13.7</v>
       </c>
     </row>
-    <row r="21" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="21" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B21" s="3">
         <v>2001</v>
       </c>
@@ -2270,10 +2590,10 @@
         <v>15</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K21" s="5">
         <v>17.7</v>
@@ -2282,10 +2602,10 @@
         <v>12.5</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N21" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O21" s="5">
         <v>100</v>
@@ -2294,7 +2614,7 @@
         <v>14.1</v>
       </c>
     </row>
-    <row r="22" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="22" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B22" s="3">
         <v>2000</v>
       </c>
@@ -2317,10 +2637,10 @@
         <v>15.5</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K22" s="4">
         <v>15.1</v>
@@ -2329,10 +2649,10 @@
         <v>13.4</v>
       </c>
       <c r="M22" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N22" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O22" s="4">
         <v>100</v>
@@ -2341,7 +2661,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="23" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="23" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B23" s="3">
         <v>1999</v>
       </c>
@@ -2364,10 +2684,10 @@
         <v>16.2</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K23" s="5">
         <v>12.6</v>
@@ -2376,10 +2696,10 @@
         <v>13.9</v>
       </c>
       <c r="M23" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N23" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O23" s="5">
         <v>100</v>
@@ -2388,7 +2708,7 @@
         <v>15.4</v>
       </c>
     </row>
-    <row r="24" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="24" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B24" s="3">
         <v>1998</v>
       </c>
@@ -2396,19 +2716,19 @@
         <v>20.2</v>
       </c>
       <c r="D24" s="4">
-        <v>16.1</v>
+        <v>16.100000000000001</v>
       </c>
       <c r="E24" s="4">
         <v>31.8</v>
       </c>
       <c r="F24" s="4">
-        <v>16.9</v>
+        <v>16.899999999999999</v>
       </c>
       <c r="G24" s="4">
         <v>26.1</v>
       </c>
       <c r="H24" s="4">
-        <v>17.1</v>
+        <v>17.100000000000001</v>
       </c>
       <c r="I24" s="4">
         <v>13.7</v>
@@ -2417,16 +2737,16 @@
         <v>14.2</v>
       </c>
       <c r="K24" s="4">
-        <v>8.3</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="L24" s="4">
         <v>15</v>
       </c>
       <c r="M24" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N24" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O24" s="4">
         <v>100</v>
@@ -2435,7 +2755,7 @@
         <v>16.2</v>
       </c>
     </row>
-    <row r="25" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="25" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B25" s="3">
         <v>1997</v>
       </c>
@@ -2449,13 +2769,13 @@
         <v>34.1</v>
       </c>
       <c r="F25" s="5">
-        <v>17.6</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="G25" s="5">
         <v>27.6</v>
       </c>
       <c r="H25" s="5">
-        <v>17.6</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="I25" s="5">
         <v>13.1</v>
@@ -2470,24 +2790,24 @@
         <v>16</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N25" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O25" s="5">
         <v>100</v>
       </c>
       <c r="P25" s="5">
-        <v>16.9</v>
-      </c>
-    </row>
-    <row r="26" s="1" customFormat="1" ht="19.7321" customHeight="1">
+        <v>16.899999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B26" s="3">
         <v>1996</v>
       </c>
       <c r="C26" s="4">
-        <v>16.6</v>
+        <v>16.600000000000001</v>
       </c>
       <c r="D26" s="4">
         <v>17.5</v>
@@ -2496,7 +2816,7 @@
         <v>35.1</v>
       </c>
       <c r="F26" s="4">
-        <v>17.9</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="G26" s="4">
         <v>28.7</v>
@@ -2517,19 +2837,19 @@
         <v>16.5</v>
       </c>
       <c r="M26" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N26" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O26" s="4">
         <v>100</v>
       </c>
       <c r="P26" s="4">
-        <v>17.1</v>
-      </c>
-    </row>
-    <row r="27" s="1" customFormat="1" ht="19.7321" customHeight="1">
+        <v>17.100000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B27" s="3">
         <v>1995</v>
       </c>
@@ -2543,7 +2863,7 @@
         <v>32.1</v>
       </c>
       <c r="F27" s="5">
-        <v>16.4</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="G27" s="5">
         <v>29.5</v>
@@ -2558,16 +2878,16 @@
         <v>13.8</v>
       </c>
       <c r="K27" s="5">
-        <v>9.2</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="L27" s="5">
         <v>15.8</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N27" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O27" s="5">
         <v>100</v>
@@ -2576,7 +2896,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="28" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B28" s="3">
         <v>1994</v>
       </c>
@@ -2608,13 +2928,13 @@
         <v>12.4</v>
       </c>
       <c r="L28" s="4">
-        <v>18.4</v>
+        <v>18.399999999999999</v>
       </c>
       <c r="M28" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N28" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O28" s="4">
         <v>100</v>
@@ -2623,7 +2943,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="29" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="29" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B29" s="3">
         <v>1993</v>
       </c>
@@ -2637,13 +2957,13 @@
         <v>32.1</v>
       </c>
       <c r="F29" s="5">
-        <v>17.9</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="G29" s="5">
         <v>32</v>
       </c>
       <c r="H29" s="5">
-        <v>17.6</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="I29" s="5">
         <v>15.5</v>
@@ -2655,13 +2975,13 @@
         <v>6.8</v>
       </c>
       <c r="L29" s="5">
-        <v>17.4</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="M29" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N29" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O29" s="5">
         <v>100</v>
@@ -2670,7 +2990,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="30" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B30" s="6">
         <v>1992</v>
       </c>
@@ -2681,7 +3001,7 @@
         <v>17</v>
       </c>
       <c r="E30" s="7">
-        <v>32.8</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="F30" s="7">
         <v>18</v>
@@ -2690,7 +3010,7 @@
         <v>35.6</v>
       </c>
       <c r="H30" s="7">
-        <v>17.4</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="I30" s="7">
         <v>17.2</v>
@@ -2702,13 +3022,13 @@
         <v>3.1</v>
       </c>
       <c r="L30" s="7">
-        <v>17.9</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="M30" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N30" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O30" s="7">
         <v>100</v>
@@ -2717,8 +3037,8 @@
         <v>16.8</v>
       </c>
     </row>
-    <row r="31" s="1" customFormat="1" ht="6.9329" customHeight="1"/>
-    <row r="32" s="1" customFormat="1" ht="96.5273" customHeight="1">
+    <row r="31" spans="2:16" s="1" customFormat="1" ht="6.95" customHeight="1"/>
+    <row r="32" spans="2:16" s="1" customFormat="1" ht="96.6" customHeight="1">
       <c r="B32" s="10" t="s">
         <v>12</v>
       </c>
@@ -2736,6 +3056,7 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="O6:P6"/>
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="B32:M32"/>
     <mergeCell ref="B6:B7"/>
@@ -2745,140 +3066,140 @@
     <mergeCell ref="I6:J6"/>
     <mergeCell ref="K6:L6"/>
     <mergeCell ref="M6:N6"/>
-    <mergeCell ref="O6:P6"/>
   </mergeCells>
-  <pageSetup paperSize="9" scale="100" orientation="portrait"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O32"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="B1:P32"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4.67767866666667" customWidth="1"/>
-    <col min="2" max="2" width="10.7125106666667" customWidth="1"/>
-    <col min="3" max="3" width="10.685892" customWidth="1"/>
-    <col min="4" max="4" width="12.7089106666667" customWidth="1"/>
-    <col min="5" max="5" width="10.6820893333333" customWidth="1"/>
-    <col min="6" max="6" width="12.7089106666667" customWidth="1"/>
-    <col min="7" max="7" width="10.6820893333333" customWidth="1"/>
-    <col min="8" max="8" width="12.7089106666667" customWidth="1"/>
-    <col min="9" max="9" width="10.6820893333333" customWidth="1"/>
-    <col min="10" max="10" width="12.7089106666667" customWidth="1"/>
-    <col min="11" max="11" width="10.6820893333333" customWidth="1"/>
-    <col min="12" max="12" width="12.7089106666667" customWidth="1"/>
-    <col min="13" max="13" width="10.6820893333333" customWidth="1"/>
-    <col min="14" max="14" width="12.7089106666667" customWidth="1"/>
-    <col min="15" max="15" width="10.6820893333333" customWidth="1"/>
-    <col min="16" max="16" width="12.7089106666667" customWidth="1"/>
+    <col min="1" max="1" width="4.7109375" customWidth="1"/>
+    <col min="2" max="3" width="10.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="10.7109375" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" customWidth="1"/>
+    <col min="15" max="15" width="10.7109375" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" ht="28.7982" customHeight="1"/>
-    <row r="2" s="1" customFormat="1" ht="31.4647" customHeight="1">
-      <c r="B2" s="8" t="s">
+    <row r="1" spans="2:16" s="1" customFormat="1" ht="28.7" customHeight="1"/>
+    <row r="2" spans="2:16" s="1" customFormat="1" ht="31.5" customHeight="1">
+      <c r="B2" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+    </row>
+    <row r="3" spans="2:16" s="1" customFormat="1" ht="14.45" customHeight="1"/>
+    <row r="4" spans="2:16" s="1" customFormat="1" ht="11.1" customHeight="1">
+      <c r="B4" s="8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:16" s="1" customFormat="1" ht="6.95" customHeight="1"/>
+    <row r="6" spans="2:16" s="1" customFormat="1" ht="24" customHeight="1">
+      <c r="B6" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="12"/>
+      <c r="I6" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="L6" s="12"/>
+      <c r="M6" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-    </row>
-    <row r="3" s="1" customFormat="1" ht="14.3991" customHeight="1"/>
-    <row r="4" s="1" customFormat="1" ht="11.1993" customHeight="1">
-      <c r="B4" s="9" t="s">
+      <c r="P6" s="12"/>
+    </row>
+    <row r="7" spans="2:16" s="1" customFormat="1" ht="24" customHeight="1">
+      <c r="B7" s="11"/>
+      <c r="C7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" s="1" customFormat="1" ht="6.9329" customHeight="1"/>
-    <row r="6" s="1" customFormat="1" ht="23.9985" customHeight="1">
-      <c r="B6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C6" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="P6" s="11"/>
-    </row>
-    <row r="7" s="1" customFormat="1" ht="23.9985" customHeight="1">
-      <c r="B7" s="2"/>
-      <c r="C7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="E7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="P7" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" s="1" customFormat="1" ht="19.7321" customHeight="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B8" s="3">
         <v>2014</v>
       </c>
       <c r="C8" s="4">
-        <v>20.4</v>
+        <v>20.399999999999999</v>
       </c>
       <c r="D8" s="4">
         <v>12.4</v>
@@ -2920,7 +3241,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="9" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B9" s="3">
         <v>2013</v>
       </c>
@@ -2937,7 +3258,7 @@
         <v>12.2</v>
       </c>
       <c r="G9" s="5">
-        <v>16.9</v>
+        <v>16.899999999999999</v>
       </c>
       <c r="H9" s="5">
         <v>11.4</v>
@@ -2955,10 +3276,10 @@
         <v>12.2</v>
       </c>
       <c r="M9" s="5">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="N9" s="5">
-        <v>9.3</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="O9" s="5">
         <v>100</v>
@@ -2967,7 +3288,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="10" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B10" s="3">
         <v>2012</v>
       </c>
@@ -3005,7 +3326,7 @@
         <v>2.5</v>
       </c>
       <c r="N10" s="4">
-        <v>9.8</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="O10" s="4">
         <v>100</v>
@@ -3014,7 +3335,7 @@
         <v>12.6</v>
       </c>
     </row>
-    <row r="11" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="11" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B11" s="3">
         <v>2011</v>
       </c>
@@ -3037,7 +3358,7 @@
         <v>11</v>
       </c>
       <c r="I11" s="5">
-        <v>17.6</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="J11" s="5">
         <v>11.1</v>
@@ -3052,7 +3373,7 @@
         <v>2.6</v>
       </c>
       <c r="N11" s="5">
-        <v>9.3</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="O11" s="5">
         <v>100</v>
@@ -3061,7 +3382,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="12" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="12" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B12" s="3">
         <v>2010</v>
       </c>
@@ -3084,10 +3405,10 @@
         <v>9.5</v>
       </c>
       <c r="I12" s="4">
-        <v>17.9</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="J12" s="4">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="K12" s="4">
         <v>45.9</v>
@@ -3099,7 +3420,7 @@
         <v>2.7</v>
       </c>
       <c r="N12" s="4">
-        <v>9.2</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="O12" s="4">
         <v>100</v>
@@ -3108,7 +3429,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="13" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="13" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B13" s="3">
         <v>2009</v>
       </c>
@@ -3119,7 +3440,7 @@
         <v>12.2</v>
       </c>
       <c r="E13" s="5">
-        <v>4.9</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="F13" s="5">
         <v>12.5</v>
@@ -3146,7 +3467,7 @@
         <v>2.7</v>
       </c>
       <c r="N13" s="5">
-        <v>9.7</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="O13" s="5">
         <v>100</v>
@@ -3155,7 +3476,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="14" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="14" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B14" s="3">
         <v>2008</v>
       </c>
@@ -3166,7 +3487,7 @@
         <v>12.5</v>
       </c>
       <c r="E14" s="4">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="F14" s="4">
         <v>12.8</v>
@@ -3202,7 +3523,7 @@
         <v>12.3</v>
       </c>
     </row>
-    <row r="15" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="15" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B15" s="3">
         <v>2007</v>
       </c>
@@ -3219,7 +3540,7 @@
         <v>13.2</v>
       </c>
       <c r="G15" s="5">
-        <v>9.2</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="H15" s="5">
         <v>12.9</v>
@@ -3240,7 +3561,7 @@
         <v>3.5</v>
       </c>
       <c r="N15" s="5">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="O15" s="5">
         <v>100</v>
@@ -3249,18 +3570,18 @@
         <v>11.9</v>
       </c>
     </row>
-    <row r="16" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="16" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B16" s="3">
         <v>2006</v>
       </c>
       <c r="C16" s="4">
-        <v>17.9</v>
+        <v>17.899999999999999</v>
       </c>
       <c r="D16" s="4">
         <v>11.7</v>
       </c>
       <c r="E16" s="4">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="F16" s="4">
         <v>13.1</v>
@@ -3296,7 +3617,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="17" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B17" s="3">
         <v>2005</v>
       </c>
@@ -3343,7 +3664,7 @@
         <v>12.6</v>
       </c>
     </row>
-    <row r="18" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="18" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B18" s="3">
         <v>2004</v>
       </c>
@@ -3372,7 +3693,7 @@
         <v>13.9</v>
       </c>
       <c r="K18" s="4">
-        <v>40.7</v>
+        <v>40.700000000000003</v>
       </c>
       <c r="L18" s="4">
         <v>13.3</v>
@@ -3390,7 +3711,7 @@
         <v>13.2</v>
       </c>
     </row>
-    <row r="19" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="19" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B19" s="3">
         <v>2003</v>
       </c>
@@ -3437,7 +3758,7 @@
         <v>13.3</v>
       </c>
     </row>
-    <row r="20" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="20" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B20" s="3">
         <v>2002</v>
       </c>
@@ -3484,7 +3805,7 @@
         <v>13.7</v>
       </c>
     </row>
-    <row r="21" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="21" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B21" s="3">
         <v>2001</v>
       </c>
@@ -3507,7 +3828,7 @@
         <v>14.3</v>
       </c>
       <c r="I21" s="5">
-        <v>9.7</v>
+        <v>9.6999999999999993</v>
       </c>
       <c r="J21" s="5">
         <v>14.6</v>
@@ -3531,12 +3852,12 @@
         <v>14.1</v>
       </c>
     </row>
-    <row r="22" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="22" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B22" s="3">
         <v>2000</v>
       </c>
       <c r="C22" s="4">
-        <v>38.3</v>
+        <v>38.299999999999997</v>
       </c>
       <c r="D22" s="4">
         <v>15.2</v>
@@ -3545,7 +3866,7 @@
         <v>7.4</v>
       </c>
       <c r="F22" s="4">
-        <v>16.1</v>
+        <v>16.100000000000001</v>
       </c>
       <c r="G22" s="4">
         <v>14.2</v>
@@ -3578,7 +3899,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="23" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="23" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B23" s="3">
         <v>1999</v>
       </c>
@@ -3589,10 +3910,10 @@
         <v>16.2</v>
       </c>
       <c r="E23" s="5">
-        <v>8.3</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="F23" s="5">
-        <v>16.4</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="G23" s="5">
         <v>15.6</v>
@@ -3601,7 +3922,7 @@
         <v>15.5</v>
       </c>
       <c r="I23" s="5">
-        <v>10.2</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="J23" s="5">
         <v>15.8</v>
@@ -3625,7 +3946,7 @@
         <v>15.4</v>
       </c>
     </row>
-    <row r="24" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="24" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B24" s="3">
         <v>1998</v>
       </c>
@@ -3636,16 +3957,16 @@
         <v>17</v>
       </c>
       <c r="E24" s="4">
-        <v>8.2</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="F24" s="4">
         <v>17.2</v>
       </c>
       <c r="G24" s="4">
-        <v>16.1</v>
+        <v>16.100000000000001</v>
       </c>
       <c r="H24" s="4">
-        <v>16.6</v>
+        <v>16.600000000000001</v>
       </c>
       <c r="I24" s="4">
         <v>12.5</v>
@@ -3672,7 +3993,7 @@
         <v>16.2</v>
       </c>
     </row>
-    <row r="25" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="25" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B25" s="3">
         <v>1997</v>
       </c>
@@ -3692,13 +4013,13 @@
         <v>13.9</v>
       </c>
       <c r="H25" s="5">
-        <v>17.6</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="I25" s="5">
         <v>11.4</v>
       </c>
       <c r="J25" s="5">
-        <v>16.9</v>
+        <v>16.899999999999999</v>
       </c>
       <c r="K25" s="5">
         <v>23.6</v>
@@ -3716,10 +4037,10 @@
         <v>100</v>
       </c>
       <c r="P25" s="5">
-        <v>16.9</v>
-      </c>
-    </row>
-    <row r="26" s="1" customFormat="1" ht="19.7321" customHeight="1">
+        <v>16.899999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B26" s="3">
         <v>1996</v>
       </c>
@@ -3739,7 +4060,7 @@
         <v>9.1</v>
       </c>
       <c r="H26" s="4">
-        <v>18.1</v>
+        <v>18.100000000000001</v>
       </c>
       <c r="I26" s="4">
         <v>11.7</v>
@@ -3763,10 +4084,10 @@
         <v>100</v>
       </c>
       <c r="P26" s="4">
-        <v>17.1</v>
-      </c>
-    </row>
-    <row r="27" s="1" customFormat="1" ht="19.7321" customHeight="1">
+        <v>17.100000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B27" s="3">
         <v>1995</v>
       </c>
@@ -3813,7 +4134,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="28" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B28" s="3">
         <v>1994</v>
       </c>
@@ -3824,7 +4145,7 @@
         <v>18</v>
       </c>
       <c r="E28" s="4">
-        <v>8.8</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="F28" s="4">
         <v>16.7</v>
@@ -3833,7 +4154,7 @@
         <v>7.3</v>
       </c>
       <c r="H28" s="4">
-        <v>16.6</v>
+        <v>16.600000000000001</v>
       </c>
       <c r="I28" s="4">
         <v>7.1</v>
@@ -3860,7 +4181,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="29" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="29" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B29" s="3">
         <v>1993</v>
       </c>
@@ -3868,7 +4189,7 @@
         <v>46.1</v>
       </c>
       <c r="D29" s="5">
-        <v>18.4</v>
+        <v>18.399999999999999</v>
       </c>
       <c r="E29" s="5">
         <v>8.5</v>
@@ -3907,7 +4228,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" s="1" customFormat="1" ht="19.7321" customHeight="1">
+    <row r="30" spans="2:16" s="1" customFormat="1" ht="19.7" customHeight="1">
       <c r="B30" s="6">
         <v>1992</v>
       </c>
@@ -3915,7 +4236,7 @@
         <v>42.5</v>
       </c>
       <c r="D30" s="7">
-        <v>18.6</v>
+        <v>18.600000000000001</v>
       </c>
       <c r="E30" s="7">
         <v>10</v>
@@ -3954,8 +4275,8 @@
         <v>16.8</v>
       </c>
     </row>
-    <row r="31" s="1" customFormat="1" ht="6.9329" customHeight="1"/>
-    <row r="32" s="1" customFormat="1" ht="96.5273" customHeight="1">
+    <row r="31" spans="2:16" s="1" customFormat="1" ht="6.95" customHeight="1"/>
+    <row r="32" spans="2:16" s="1" customFormat="1" ht="96.6" customHeight="1">
       <c r="B32" s="10" t="s">
         <v>12</v>
       </c>
@@ -3973,6 +4294,7 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="O6:P6"/>
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="B32:M32"/>
     <mergeCell ref="B6:B7"/>
@@ -3982,9 +4304,9 @@
     <mergeCell ref="I6:J6"/>
     <mergeCell ref="K6:L6"/>
     <mergeCell ref="M6:N6"/>
-    <mergeCell ref="O6:P6"/>
   </mergeCells>
-  <pageSetup paperSize="9" scale="100" orientation="portrait"/>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
</xml_diff>